<commit_message>
add: update C2-W3 Practice Challenge Excel file with new content
</commit_message>
<xml_diff>
--- a/02-intermediate-1/material_curso/modulo-03/challenge/C2-W3-Practice-Challenge.xlsx
+++ b/02-intermediate-1/material_curso/modulo-03/challenge/C2-W3-Practice-Challenge.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Proyectos\ExcelLearning\02-intermediate-1\material_curso\modulo-03\challenge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1980674-0353-4FFE-8293-A3BB2EC13EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7DA429-9D43-4EF6-BA37-E35BBCA3597F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="687" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4620" yWindow="4620" windowWidth="14430" windowHeight="7755" tabRatio="687" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="17" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <definedName name="Quoted_price_to_the_customer">'Project-Data'!$H$6:$H$65</definedName>
     <definedName name="Total_receipts">'Project-Data'!$M$6:$M$65</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -2369,28 +2369,28 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="24" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="9" fontId="24" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="9" fontId="24" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2417,28 +2417,28 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="9" fontId="24" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="9" fontId="24" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="9" fontId="24" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -4781,7 +4781,7 @@
       <c r="C1" s="19"/>
       <c r="D1" s="20"/>
       <c r="E1" s="20"/>
-      <c r="F1" s="67" t="s">
+      <c r="F1" s="79" t="s">
         <v>51</v>
       </c>
       <c r="G1" s="20"/>
@@ -4800,7 +4800,7 @@
       <c r="L1" s="22">
         <v>0.3</v>
       </c>
-      <c r="M1" s="64" t="s">
+      <c r="M1" s="76" t="s">
         <v>52</v>
       </c>
       <c r="N1" s="85" t="s">
@@ -4816,7 +4816,7 @@
       <c r="C2" s="19"/>
       <c r="D2" s="20"/>
       <c r="E2" s="20"/>
-      <c r="F2" s="68"/>
+      <c r="F2" s="80"/>
       <c r="G2" s="20"/>
       <c r="H2" s="23" t="s">
         <v>26</v>
@@ -4833,7 +4833,7 @@
       <c r="L2" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="65"/>
+      <c r="M2" s="77"/>
       <c r="N2" s="86"/>
       <c r="O2" s="86"/>
       <c r="P2" s="31"/>
@@ -4843,7 +4843,7 @@
       <c r="C3"/>
       <c r="D3" s="20"/>
       <c r="E3" s="20"/>
-      <c r="F3" s="69"/>
+      <c r="F3" s="81"/>
       <c r="G3" s="20"/>
       <c r="H3" s="53" t="s">
         <v>56</v>
@@ -4860,7 +4860,7 @@
       <c r="L3" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="M3" s="66"/>
+      <c r="M3" s="78"/>
       <c r="N3" s="87"/>
       <c r="O3" s="87"/>
       <c r="P3" s="31"/>
@@ -4992,10 +4992,10 @@
       <c r="Q6" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="R6" s="76" t="s">
+      <c r="R6" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="S6" s="79">
+      <c r="S6" s="67">
         <f>SUM(Project_cost)</f>
         <v>2441700</v>
       </c>
@@ -5054,8 +5054,8 @@
         <v>37800</v>
       </c>
       <c r="Q7" s="74"/>
-      <c r="R7" s="77"/>
-      <c r="S7" s="80"/>
+      <c r="R7" s="65"/>
+      <c r="S7" s="68"/>
       <c r="T7" s="71"/>
     </row>
     <row r="8" spans="2:21" ht="15.75" thickBot="1">
@@ -5107,8 +5107,8 @@
         <v>79200</v>
       </c>
       <c r="Q8" s="75"/>
-      <c r="R8" s="78"/>
-      <c r="S8" s="81"/>
+      <c r="R8" s="66"/>
+      <c r="S8" s="69"/>
       <c r="T8" s="72"/>
     </row>
     <row r="9" spans="2:21">
@@ -5162,10 +5162,10 @@
       <c r="Q9" s="73" t="s">
         <v>58</v>
       </c>
-      <c r="R9" s="76" t="s">
+      <c r="R9" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="S9" s="79">
+      <c r="S9" s="67">
         <f>AVERAGE(Project_cost)</f>
         <v>40695</v>
       </c>
@@ -5223,8 +5223,8 @@
         <v>63000</v>
       </c>
       <c r="Q10" s="74"/>
-      <c r="R10" s="77"/>
-      <c r="S10" s="80"/>
+      <c r="R10" s="65"/>
+      <c r="S10" s="68"/>
       <c r="T10" s="71"/>
     </row>
     <row r="11" spans="2:21" ht="15" customHeight="1" thickBot="1">
@@ -5276,8 +5276,8 @@
         <v>27900</v>
       </c>
       <c r="Q11" s="75"/>
-      <c r="R11" s="78"/>
-      <c r="S11" s="81"/>
+      <c r="R11" s="66"/>
+      <c r="S11" s="69"/>
       <c r="T11" s="72"/>
     </row>
     <row r="12" spans="2:21" ht="15" customHeight="1">
@@ -5331,10 +5331,10 @@
       <c r="Q12" s="73" t="s">
         <v>59</v>
       </c>
-      <c r="R12" s="76" t="s">
+      <c r="R12" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="S12" s="79">
+      <c r="S12" s="67">
         <f>MAX(Project_cost)</f>
         <v>92700</v>
       </c>
@@ -5392,8 +5392,8 @@
         <v>47700</v>
       </c>
       <c r="Q13" s="74"/>
-      <c r="R13" s="77"/>
-      <c r="S13" s="80"/>
+      <c r="R13" s="65"/>
+      <c r="S13" s="68"/>
       <c r="T13" s="71"/>
     </row>
     <row r="14" spans="2:21" ht="15.75" thickBot="1">
@@ -5445,8 +5445,8 @@
         <v>63000</v>
       </c>
       <c r="Q14" s="75"/>
-      <c r="R14" s="78"/>
-      <c r="S14" s="81"/>
+      <c r="R14" s="66"/>
+      <c r="S14" s="69"/>
       <c r="T14" s="72"/>
     </row>
     <row r="15" spans="2:21">
@@ -5500,10 +5500,10 @@
       <c r="Q15" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="R15" s="76" t="s">
+      <c r="R15" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="S15" s="79">
+      <c r="S15" s="67">
         <f>MIN(Project_cost)</f>
         <v>6300</v>
       </c>
@@ -5561,8 +5561,8 @@
         <v>8100</v>
       </c>
       <c r="Q16" s="74"/>
-      <c r="R16" s="77"/>
-      <c r="S16" s="80"/>
+      <c r="R16" s="65"/>
+      <c r="S16" s="68"/>
       <c r="T16" s="71"/>
     </row>
     <row r="17" spans="2:20" ht="15.75" thickBot="1">
@@ -5614,8 +5614,8 @@
         <v>14400</v>
       </c>
       <c r="Q17" s="75"/>
-      <c r="R17" s="78"/>
-      <c r="S17" s="81"/>
+      <c r="R17" s="66"/>
+      <c r="S17" s="69"/>
       <c r="T17" s="72"/>
     </row>
     <row r="18" spans="2:20">
@@ -7985,14 +7985,6 @@
     <sortCondition ref="C6:C65"/>
   </sortState>
   <mergeCells count="21">
-    <mergeCell ref="R12:R14"/>
-    <mergeCell ref="S12:S14"/>
-    <mergeCell ref="T12:T14"/>
-    <mergeCell ref="Q15:Q17"/>
-    <mergeCell ref="R15:R17"/>
-    <mergeCell ref="S15:S17"/>
-    <mergeCell ref="T15:T17"/>
-    <mergeCell ref="Q12:Q14"/>
     <mergeCell ref="M1:M3"/>
     <mergeCell ref="F1:F3"/>
     <mergeCell ref="T6:T8"/>
@@ -8006,6 +7998,14 @@
     <mergeCell ref="I4:M4"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="O1:O3"/>
+    <mergeCell ref="R12:R14"/>
+    <mergeCell ref="S12:S14"/>
+    <mergeCell ref="T12:T14"/>
+    <mergeCell ref="Q15:Q17"/>
+    <mergeCell ref="R15:R17"/>
+    <mergeCell ref="S15:S17"/>
+    <mergeCell ref="T15:T17"/>
+    <mergeCell ref="Q12:Q14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="256" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>